<commit_message>
Updated the structure for non trainee's letters
</commit_message>
<xml_diff>
--- a/samples/Appointment Letter and Employment Agreement - JaipurBangalore.xlsx
+++ b/samples/Appointment Letter and Employment Agreement - JaipurBangalore.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wordToPdf\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DAA86E5-5350-4D92-8FC6-AFFEEA5DBBDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30D2EE2-FDF0-4397-95A9-669B7B2F39D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{6E3B9890-34E2-4B4A-8915-E48360C036C6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Date of Joining</t>
   </si>
@@ -97,6 +97,30 @@
   </si>
   <si>
     <t>Junior Software Engineer</t>
+  </si>
+  <si>
+    <t>Trainee Address line1</t>
+  </si>
+  <si>
+    <t>Trainee Address line2</t>
+  </si>
+  <si>
+    <t>Trainee Address line3</t>
+  </si>
+  <si>
+    <t>Flat no, 305, Rachana Ashwini</t>
+  </si>
+  <si>
+    <t>Apartment, Jagdish Nagar,</t>
+  </si>
+  <si>
+    <t>Katolroad,Nagpur, Mahaeashtra-440013</t>
+  </si>
+  <si>
+    <t>115, Sai Sumukha Apartment, FN 504</t>
+  </si>
+  <si>
+    <t>layout,Mariyappanapalya VTC ,Bangalore Distrit, Kartnataka-560056</t>
   </si>
 </sst>
 </file>
@@ -490,20 +514,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C9EAFDC-0661-4263-8911-B2C3A4238E1D}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="72.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="71.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="71.7109375" customWidth="1"/>
+    <col min="5" max="5" width="71.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="72.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -511,99 +539,123 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>18</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>16</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>45838</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2">
+      <c r="G2">
         <v>8947880022</v>
       </c>
-      <c r="E2" t="s">
+      <c r="H2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="1">
+      <c r="I2" s="1">
         <v>45838</v>
       </c>
-      <c r="G2" t="s">
+      <c r="J2" t="s">
         <v>9</v>
       </c>
-      <c r="H2" t="s">
+      <c r="K2" t="s">
         <v>12</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
+      <c r="M2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>45874</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D3">
+      <c r="G3">
         <v>2938475673</v>
       </c>
-      <c r="E3" t="s">
+      <c r="H3" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="1">
+      <c r="I3" s="1">
         <v>45874</v>
       </c>
-      <c r="G3" t="s">
+      <c r="J3" t="s">
         <v>13</v>
       </c>
-      <c r="H3" t="s">
+      <c r="K3" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s">
+      <c r="L3" t="s">
         <v>21</v>
       </c>
-      <c r="J3" t="s">
+      <c r="M3" t="s">
         <v>22</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{32B693B5-0E31-49A9-BE78-637BEBFB5C76}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{F1EFB166-B36A-4E91-B8C9-FF1CEB5602E3}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{32B693B5-0E31-49A9-BE78-637BEBFB5C76}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{F1EFB166-B36A-4E91-B8C9-FF1CEB5602E3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>